<commit_message>
--IMPLEMENTACION DE CONDICIONAL PARA EVITAR ESCRIBIR CARACTERES VACIOS EN EL CODIGO DE LA FACTURA Y EN SU VENCIMIENTO, YA QUE EL SISTEMA SIDIF NO LO RECONOCE, CAMBIANDOLO POR UN CONDICIONAL TERNARIO EL CUAL EN CASO DE QUE SEA UN EMPTY STRING, ASIGNE UN NULL A LOS VALORES
--CAMBIOS MENORES EN EL FORMATO DE LA PLANTILLA DE EXPORTACION
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/PLANTILLA.xlsx
+++ b/Control de Facturas/Assets/Plantillas/PLANTILLA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B98522-6375-42A2-9B6A-AC20A76D52D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B5FF04-54EC-42EE-80D0-2A3B94EDDA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="900" xr2:uid="{D9D33F21-ED07-47A1-8533-367C0DEB1D0B}"/>
+    <workbookView xWindow="-20610" yWindow="-60" windowWidth="20730" windowHeight="11040" tabRatio="900" xr2:uid="{D9D33F21-ED07-47A1-8533-367C0DEB1D0B}"/>
   </bookViews>
   <sheets>
     <sheet name="Cabecera-Cpte" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId9"/>
+    <pivotCache cacheId="10" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -2909,7 +2909,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="62">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -3047,32 +3047,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -3111,30 +3085,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -3296,54 +3246,10 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -3369,163 +3275,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -3554,73 +3305,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -3698,18 +3382,14 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="164">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -3718,7 +3398,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3728,144 +3408,29 @@
     <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="29" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" pivotButton="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" pivotButton="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="2" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3873,279 +3438,149 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="32" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="27" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="27" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="27" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="27" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="27" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="61" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="31" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="32" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="16" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="32" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="42" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -4562,7 +3997,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FB68EB4-76D3-458C-A6F3-4728B0F719D5}" name="Tabla dinámica2" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FB68EB4-76D3-458C-A6F3-4728B0F719D5}" name="Tabla dinámica2" cacheId="10" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
   <location ref="A3:L31" firstHeaderRow="2" firstDataRow="2" firstDataCol="6"/>
   <pivotFields count="7">
     <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
@@ -5176,473 +4611,452 @@
   <dimension ref="A1:AM5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="42" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" style="42" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" style="42" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" style="46" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" style="46" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" style="46" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.140625" style="42" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="42" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" style="66" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" style="42" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="5.85546875" style="46" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12" style="46" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.28515625" style="46" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.5703125" style="163" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="37.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="5" style="2" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="3.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="4" style="2" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="22.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="4" style="2" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="4.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="3.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="3.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="7" style="2" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="4.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="2.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="8.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="4.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="4.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="6.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="23" style="2" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="30.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="12.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="18.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="79" max="80" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="23.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="25.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="35.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="2.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="9.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="12.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="18.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="23.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="25.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="34.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="16.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="2.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="9.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="133" max="135" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="136" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="14" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" style="28" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" style="36" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.28515625" style="36" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" style="36" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="28" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="28" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.85546875" style="36" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="7.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12" style="36" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.28515625" style="36" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="16.5703125" style="42" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="37.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="5" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="3.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="4" style="29" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="20.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="7.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="18.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="22.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="4" style="29" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="3.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="3.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="7" style="29" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="4.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="6.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="23" style="29" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="14" style="29" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="79" max="80" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="23.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="25.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="35.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="16.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="23.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="25.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="34.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="16.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="14.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="132" max="132" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="133" max="135" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="136" max="16384" width="11.42578125" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="84" t="s">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.2">
+      <c r="A1" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
-      <c r="I1" s="86"/>
-      <c r="J1" s="86"/>
-      <c r="K1" s="86"/>
-      <c r="L1" s="86"/>
-      <c r="M1" s="86"/>
-      <c r="N1" s="86"/>
-      <c r="O1" s="85"/>
-      <c r="P1" s="85"/>
-      <c r="Q1" s="85"/>
-      <c r="R1" s="85"/>
-      <c r="S1" s="85"/>
-      <c r="T1" s="85"/>
-      <c r="U1" s="85"/>
-      <c r="V1" s="85"/>
-      <c r="W1" s="85"/>
-      <c r="X1" s="85"/>
-      <c r="Y1" s="85"/>
-      <c r="Z1" s="85"/>
-      <c r="AA1" s="85"/>
-      <c r="AB1" s="85"/>
-      <c r="AC1" s="85"/>
-      <c r="AD1" s="85"/>
-      <c r="AE1" s="85"/>
-      <c r="AF1" s="85"/>
-      <c r="AG1" s="85"/>
-      <c r="AH1" s="85"/>
-      <c r="AI1" s="85"/>
-      <c r="AJ1" s="87"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
     </row>
     <row r="2" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="77"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="93" t="s">
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="88" t="s">
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="88"/>
-      <c r="Q2" s="76" t="s">
+      <c r="P2" s="45"/>
+      <c r="Q2" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="R2" s="77"/>
-      <c r="S2" s="77"/>
-      <c r="T2" s="78"/>
-      <c r="U2" s="76" t="s">
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="V2" s="77"/>
-      <c r="W2" s="78"/>
-      <c r="X2" s="76" t="s">
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="Y2" s="77"/>
-      <c r="Z2" s="77"/>
-      <c r="AA2" s="101"/>
-      <c r="AB2" s="103" t="s">
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="43"/>
+      <c r="AA2" s="43"/>
+      <c r="AB2" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="AC2" s="76" t="s">
+      <c r="AC2" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="AD2" s="77"/>
-      <c r="AE2" s="101"/>
-      <c r="AF2" s="99" t="s">
+      <c r="AD2" s="43"/>
+      <c r="AE2" s="43"/>
+      <c r="AF2" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="AG2" s="77"/>
-      <c r="AH2" s="78"/>
-      <c r="AI2" s="159" t="s">
+      <c r="AG2" s="43"/>
+      <c r="AH2" s="43"/>
+      <c r="AI2" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="AJ2" s="91" t="s">
+      <c r="AJ2" s="43" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:39" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="79"/>
-      <c r="B3" s="80"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="82" t="s">
+      <c r="A3" s="43"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="79" t="s">
+      <c r="E3" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="80"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="43" t="s">
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="96" t="s">
+      <c r="I3" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="J3" s="97"/>
-      <c r="K3" s="47" t="s">
+      <c r="J3" s="43"/>
+      <c r="K3" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
-      <c r="N3" s="82" t="s">
+      <c r="L3" s="27"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="O3" s="89" t="s">
+      <c r="O3" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="P3" s="90"/>
-      <c r="Q3" s="79"/>
-      <c r="R3" s="80"/>
-      <c r="S3" s="80"/>
-      <c r="T3" s="81"/>
-      <c r="U3" s="79"/>
-      <c r="V3" s="80"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="79"/>
-      <c r="Y3" s="80"/>
-      <c r="Z3" s="80"/>
-      <c r="AA3" s="102"/>
-      <c r="AB3" s="104"/>
-      <c r="AC3" s="79"/>
-      <c r="AD3" s="80"/>
-      <c r="AE3" s="102"/>
-      <c r="AF3" s="100"/>
-      <c r="AG3" s="80"/>
-      <c r="AH3" s="81"/>
-      <c r="AI3" s="160"/>
-      <c r="AJ3" s="92"/>
-    </row>
-    <row r="4" spans="1:39" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
+      <c r="P3" s="45"/>
+      <c r="Q3" s="43"/>
+      <c r="R3" s="43"/>
+      <c r="S3" s="43"/>
+      <c r="T3" s="43"/>
+      <c r="U3" s="43"/>
+      <c r="V3" s="43"/>
+      <c r="W3" s="43"/>
+      <c r="X3" s="43"/>
+      <c r="Y3" s="43"/>
+      <c r="Z3" s="43"/>
+      <c r="AA3" s="43"/>
+      <c r="AB3" s="43"/>
+      <c r="AC3" s="43"/>
+      <c r="AD3" s="43"/>
+      <c r="AE3" s="43"/>
+      <c r="AF3" s="43"/>
+      <c r="AG3" s="43"/>
+      <c r="AH3" s="43"/>
+      <c r="AI3" s="46"/>
+      <c r="AJ3" s="43"/>
+    </row>
+    <row r="4" spans="1:39" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="83"/>
-      <c r="E4" s="39" t="s">
+      <c r="D4" s="43"/>
+      <c r="E4" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="50" t="s">
+      <c r="F4" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="50" t="s">
+      <c r="G4" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="44" t="s">
+      <c r="H4" s="36" t="s">
         <v>79</v>
       </c>
-      <c r="I4" s="44" t="s">
+      <c r="I4" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="J4" s="44" t="s">
+      <c r="J4" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="K4" s="51" t="s">
+      <c r="K4" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="52" t="s">
+      <c r="L4" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="51" t="s">
+      <c r="M4" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="N4" s="83"/>
-      <c r="O4" s="53" t="s">
+      <c r="N4" s="43"/>
+      <c r="O4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="50" t="s">
+      <c r="P4" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="54" t="s">
+      <c r="Q4" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="R4" s="54" t="s">
+      <c r="R4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="S4" s="55" t="s">
+      <c r="S4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="T4" s="39" t="s">
+      <c r="T4" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="U4" s="56" t="s">
+      <c r="U4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="V4" s="56" t="s">
+      <c r="V4" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="W4" s="56" t="s">
+      <c r="W4" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="X4" s="56" t="s">
+      <c r="X4" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="Y4" s="56" t="s">
+      <c r="Y4" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="Z4" s="57" t="s">
+      <c r="Z4" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="AA4" s="56" t="s">
+      <c r="AA4" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="AB4" s="104"/>
-      <c r="AC4" s="53" t="s">
+      <c r="AB4" s="43"/>
+      <c r="AC4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AD4" s="53" t="s">
+      <c r="AD4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="AE4" s="53" t="s">
+      <c r="AE4" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="AF4" s="58" t="s">
+      <c r="AF4" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="AG4" s="58" t="s">
+      <c r="AG4" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="AH4" s="53" t="s">
+      <c r="AH4" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="AI4" s="161" t="s">
+      <c r="AI4" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="AJ4" s="92"/>
-      <c r="AK4" s="4" t="s">
+      <c r="AJ4" s="43"/>
+      <c r="AK4" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="AL4" s="4" t="s">
+      <c r="AL4" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="AM4" s="4" t="s">
+      <c r="AM4" s="29" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A5" s="40">
+      <c r="A5" s="28">
         <v>326</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="41">
+      <c r="C5" s="29">
         <f ca="1">YEAR(TODAY())</f>
         <v>2026</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="E5" s="41" t="s">
+      <c r="E5" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="60"/>
-      <c r="L5" s="60"/>
-      <c r="M5" s="61"/>
-      <c r="N5" s="62"/>
-      <c r="O5" s="41" t="s">
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="P5" s="40"/>
-      <c r="Q5" s="41"/>
-      <c r="R5" s="41"/>
-      <c r="S5" s="41"/>
-      <c r="T5" s="41"/>
-      <c r="U5" s="41"/>
-      <c r="V5" s="41"/>
-      <c r="W5" s="41"/>
-      <c r="X5" s="41" t="s">
+      <c r="X5" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="Y5" s="41"/>
-      <c r="Z5" s="63"/>
-      <c r="AA5" s="36">
+      <c r="AA5" s="29">
         <v>1</v>
       </c>
-      <c r="AB5" s="64" t="s">
+      <c r="AB5" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="AC5" s="41"/>
-      <c r="AD5" s="41"/>
-      <c r="AE5" s="41"/>
-      <c r="AF5" s="61"/>
-      <c r="AG5" s="61"/>
-      <c r="AH5" s="65"/>
-      <c r="AI5" s="162"/>
-      <c r="AJ5" s="65"/>
-      <c r="AK5" s="36"/>
-      <c r="AL5" s="36"/>
-      <c r="AM5" s="36">
+      <c r="AF5" s="38"/>
+      <c r="AG5" s="38"/>
+      <c r="AH5" s="30"/>
+      <c r="AI5" s="40"/>
+      <c r="AJ5" s="30"/>
+      <c r="AM5" s="29">
         <f>LEN(AJ5)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="X2:AA3"/>
-    <mergeCell ref="U2:W3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="N3:N4"/>
     <mergeCell ref="A1:AJ1"/>
     <mergeCell ref="A2:C3"/>
     <mergeCell ref="O2:P2"/>
@@ -5656,6 +5070,10 @@
     <mergeCell ref="AF2:AH3"/>
     <mergeCell ref="AC2:AE3"/>
     <mergeCell ref="AB2:AB4"/>
+    <mergeCell ref="X2:AA3"/>
+    <mergeCell ref="U2:W3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="N3:N4"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="AM1:AM1048576">
@@ -5681,76 +5099,76 @@
     <col min="4" max="4" width="4.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="114" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="I1" s="114"/>
-      <c r="J1" s="114"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="106"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="110" t="s">
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="111"/>
-      <c r="F2" s="110" t="s">
+      <c r="E2" s="53"/>
+      <c r="F2" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="111"/>
-      <c r="H2" s="112" t="s">
+      <c r="G2" s="53"/>
+      <c r="H2" s="54" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="115" t="s">
+      <c r="I2" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="117" t="s">
+      <c r="J2" s="59" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="113"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="118"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5776,111 +5194,111 @@
   <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" style="29" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.140625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="5.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" style="4"/>
-    <col min="13" max="13" width="14.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" style="4" customWidth="1"/>
-    <col min="16" max="16" width="13.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="11.42578125" style="4"/>
+    <col min="1" max="1" width="5.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" style="29" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" style="28" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.140625" style="29" customWidth="1"/>
+    <col min="10" max="10" width="5.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" style="29"/>
+    <col min="13" max="13" width="14.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" style="29" customWidth="1"/>
+    <col min="16" max="16" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14" style="29" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="11.42578125" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="107" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="61" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-      <c r="R1" s="122"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
     </row>
     <row r="2" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="106"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="110" t="s">
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="111"/>
-      <c r="F2" s="110" t="s">
+      <c r="E2" s="61"/>
+      <c r="F2" s="61" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="111"/>
-      <c r="H2" s="129" t="s">
+      <c r="G2" s="61"/>
+      <c r="H2" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="131" t="s">
+      <c r="I2" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="123" t="s">
+      <c r="J2" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="K2" s="124"/>
-      <c r="L2" s="124"/>
-      <c r="M2" s="125"/>
-      <c r="N2" s="131" t="s">
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="119" t="s">
+      <c r="O2" s="62" t="s">
         <v>66</v>
       </c>
-      <c r="P2" s="126" t="s">
+      <c r="P2" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="127"/>
-      <c r="R2" s="128"/>
-    </row>
-    <row r="3" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="Q2" s="64"/>
+      <c r="R2" s="64"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="130"/>
-      <c r="I3" s="132"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
       <c r="J3" s="33" t="s">
         <v>57</v>
       </c>
@@ -5893,66 +5311,66 @@
       <c r="M3" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="N3" s="132"/>
-      <c r="O3" s="120"/>
-      <c r="P3" s="34" t="s">
+      <c r="N3" s="64"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="34" t="s">
+      <c r="Q3" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="34" t="s">
+      <c r="R3" s="33" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="str">
+      <c r="A4" s="29" t="str">
         <f>'Cabecera-Cpte'!E5</f>
         <v>B</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="28">
         <f>'Cabecera-Cpte'!F5</f>
         <v>0</v>
       </c>
-      <c r="C4" s="29">
+      <c r="C4" s="28">
         <f>'Cabecera-Cpte'!G5</f>
         <v>0</v>
       </c>
-      <c r="D4" s="4" t="str">
+      <c r="D4" s="29" t="str">
         <f>'Cabecera-Cpte'!O5</f>
         <v>CUI</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="28">
         <f>'Cabecera-Cpte'!P5</f>
         <v>0</v>
       </c>
-      <c r="F4" s="31">
+      <c r="F4" s="34">
         <f>'Cabecera-Cpte'!K5</f>
         <v>0</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="34">
         <f>'Cabecera-Cpte'!L5</f>
         <v>0</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="29">
         <v>3</v>
       </c>
       <c r="K4" s="35">
         <v>1</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="29">
         <v>1</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="29">
         <v>0</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="29">
         <v>1</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="29">
         <f>'Cabecera-Cpte'!AI5</f>
         <v>0</v>
       </c>
@@ -5984,351 +5402,341 @@
   <dimension ref="A1:AJ4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="3.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="3.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="4" style="4" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="4.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="4.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="6.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="16384" width="11.42578125" style="4"/>
+    <col min="1" max="1" width="5.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="23" style="28" customWidth="1"/>
+    <col min="4" max="4" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23" style="29" customWidth="1"/>
+    <col min="6" max="7" width="23" style="28" customWidth="1"/>
+    <col min="8" max="8" width="8.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="29" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9" style="29" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="8.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="4" style="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8" style="29" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="6.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="23" style="29" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="17.7109375" style="42" bestFit="1" customWidth="1"/>
+    <col min="37" max="16384" width="11.42578125" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="142" t="s">
+    <row r="1" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="139" t="s">
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="140"/>
-      <c r="J1" s="140"/>
-      <c r="K1" s="140"/>
-      <c r="L1" s="140"/>
-      <c r="M1" s="140"/>
-      <c r="N1" s="140"/>
-      <c r="O1" s="140"/>
-      <c r="P1" s="140"/>
-      <c r="Q1" s="140"/>
-      <c r="R1" s="140"/>
-      <c r="S1" s="140"/>
-      <c r="T1" s="140"/>
-      <c r="U1" s="140"/>
-      <c r="V1" s="140"/>
-      <c r="W1" s="140"/>
-      <c r="X1" s="140"/>
-      <c r="Y1" s="140"/>
-      <c r="Z1" s="140"/>
-      <c r="AA1" s="140"/>
-      <c r="AB1" s="140"/>
-      <c r="AC1" s="140"/>
-      <c r="AD1" s="140"/>
-      <c r="AE1" s="140"/>
-      <c r="AF1" s="140"/>
-      <c r="AG1" s="140"/>
-      <c r="AH1" s="140"/>
-      <c r="AI1" s="140"/>
-      <c r="AJ1" s="141"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
     </row>
     <row r="2" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="133" t="s">
+      <c r="A2" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="89" t="s">
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="90"/>
-      <c r="F2" s="89" t="s">
+      <c r="E2" s="45"/>
+      <c r="F2" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="90"/>
-      <c r="H2" s="135" t="s">
+      <c r="G2" s="45"/>
+      <c r="H2" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="I2" s="135" t="s">
+      <c r="I2" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="J2" s="81" t="s">
+      <c r="J2" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98" t="s">
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="N2" s="98" t="s">
+      <c r="N2" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="98" t="s">
+      <c r="O2" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="98"/>
-      <c r="R2" s="98"/>
-      <c r="S2" s="98"/>
-      <c r="T2" s="98" t="s">
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="98" t="s">
+      <c r="U2" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="V2" s="98"/>
-      <c r="W2" s="98"/>
-      <c r="X2" s="98"/>
-      <c r="Y2" s="135" t="s">
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="Z2" s="135" t="s">
+      <c r="Z2" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="AA2" s="135" t="s">
+      <c r="AA2" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="AB2" s="137" t="s">
+      <c r="AB2" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="AC2" s="137" t="s">
+      <c r="AC2" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="AD2" s="135" t="s">
+      <c r="AD2" s="45" t="s">
         <v>74</v>
       </c>
-      <c r="AE2" s="135" t="s">
+      <c r="AE2" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="AF2" s="135" t="s">
+      <c r="AF2" s="45" t="s">
         <v>27</v>
       </c>
-      <c r="AG2" s="135" t="s">
+      <c r="AG2" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="AH2" s="135" t="s">
+      <c r="AH2" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="AI2" s="135" t="s">
+      <c r="AI2" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="AJ2" s="145" t="s">
+      <c r="AJ2" s="65" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:36" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="67" t="s">
+    <row r="3" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="68" t="s">
+      <c r="C3" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="69" t="s">
+      <c r="D3" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="67" t="s">
+      <c r="E3" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="70" t="s">
+      <c r="F3" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="71" t="s">
+      <c r="G3" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="147"/>
-      <c r="I3" s="147"/>
-      <c r="J3" s="72" t="s">
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="73" t="s">
+      <c r="K3" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="L3" s="73" t="s">
+      <c r="L3" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="134"/>
-      <c r="N3" s="134"/>
-      <c r="O3" s="74" t="s">
+      <c r="M3" s="43"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="P3" s="74" t="s">
+      <c r="P3" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="T3" s="134"/>
-      <c r="U3" s="74" t="s">
+      <c r="T3" s="43"/>
+      <c r="U3" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="V3" s="74" t="s">
+      <c r="V3" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="W3" s="74" t="s">
+      <c r="W3" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="X3" s="74" t="s">
+      <c r="X3" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="Y3" s="136"/>
-      <c r="Z3" s="136"/>
-      <c r="AA3" s="136"/>
-      <c r="AB3" s="138"/>
-      <c r="AC3" s="138"/>
-      <c r="AD3" s="136"/>
-      <c r="AE3" s="136"/>
-      <c r="AF3" s="136"/>
-      <c r="AG3" s="136"/>
-      <c r="AH3" s="136"/>
-      <c r="AI3" s="136"/>
-      <c r="AJ3" s="146"/>
+      <c r="Y3" s="45"/>
+      <c r="Z3" s="45"/>
+      <c r="AA3" s="45"/>
+      <c r="AB3" s="45"/>
+      <c r="AC3" s="45"/>
+      <c r="AD3" s="45"/>
+      <c r="AE3" s="45"/>
+      <c r="AF3" s="45"/>
+      <c r="AG3" s="45"/>
+      <c r="AH3" s="45"/>
+      <c r="AI3" s="45"/>
+      <c r="AJ3" s="65"/>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="str">
+      <c r="A4" s="29" t="str">
         <f>'Cabecera-Cpte'!E5</f>
         <v>B</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="28">
         <f>'Cabecera-Cpte'!F5</f>
         <v>0</v>
       </c>
-      <c r="C4" s="29">
+      <c r="C4" s="28">
         <f>'Cabecera-Cpte'!G5</f>
         <v>0</v>
       </c>
-      <c r="D4" s="4" t="str">
+      <c r="D4" s="29" t="str">
         <f>'Cabecera-Cpte'!O5</f>
         <v>CUI</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="29">
         <f>'Cabecera-Cpte'!P5</f>
         <v>0</v>
       </c>
-      <c r="F4" s="31">
+      <c r="F4" s="34">
         <f>'Cabecera-Cpte'!K5</f>
         <v>0</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="34">
         <f>'Cabecera-Cpte'!L5</f>
         <v>0</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="29">
         <v>41</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="29">
         <v>4</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="29">
         <v>0</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="29">
         <f>'Cabecera-Cpte'!A5</f>
         <v>326</v>
       </c>
-      <c r="N4" s="4">
-        <f>'Cabecera-Cpte'!AK5</f>
+      <c r="O4" s="29">
+        <v>1</v>
+      </c>
+      <c r="P4" s="29">
         <v>0</v>
       </c>
-      <c r="O4" s="4">
+      <c r="Q4" s="29">
+        <v>0</v>
+      </c>
+      <c r="R4" s="29">
         <v>1</v>
       </c>
-      <c r="P4" s="4">
+      <c r="S4" s="29">
         <v>0</v>
       </c>
-      <c r="Q4" s="4">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4">
-        <v>1</v>
-      </c>
-      <c r="S4" s="4">
-        <v>0</v>
-      </c>
-      <c r="T4" s="4">
-        <f>'Cabecera-Cpte'!AL5</f>
-        <v>0</v>
-      </c>
-      <c r="U4" s="4">
+      <c r="U4" s="29">
         <f>'Detalle Cpte FacGS'!J4</f>
         <v>3</v>
       </c>
-      <c r="V4" s="4">
+      <c r="V4" s="29">
         <f>'Detalle Cpte FacGS'!K4</f>
         <v>1</v>
       </c>
-      <c r="W4" s="4">
+      <c r="W4" s="29">
         <f>'Detalle Cpte FacGS'!L4</f>
         <v>1</v>
       </c>
-      <c r="X4" s="4">
+      <c r="X4" s="29">
         <f>'Detalle Cpte FacGS'!M4</f>
         <v>0</v>
       </c>
-      <c r="Y4" s="4">
+      <c r="Y4" s="29">
         <v>11</v>
       </c>
-      <c r="Z4" s="4">
+      <c r="Z4" s="29">
         <v>1</v>
       </c>
-      <c r="AB4" s="4">
+      <c r="AB4" s="29">
         <v>0</v>
       </c>
-      <c r="AC4" s="4">
+      <c r="AC4" s="29">
         <v>0</v>
       </c>
-      <c r="AE4" s="4" t="s">
+      <c r="AE4" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="AF4" s="4" t="s">
+      <c r="AF4" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="AG4" s="4" t="s">
+      <c r="AG4" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="AH4" s="4">
+      <c r="AH4" s="29">
         <v>0</v>
       </c>
-      <c r="AJ4" s="75">
+      <c r="AJ4" s="42">
         <f>'Cabecera-Cpte'!AI5</f>
         <v>0</v>
       </c>
@@ -6387,70 +5795,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="148"/>
-      <c r="H1" s="151" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="152"/>
-      <c r="J1" s="152"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="106"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="110" t="s">
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="111"/>
-      <c r="F2" s="110" t="s">
+      <c r="E2" s="53"/>
+      <c r="F2" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="111"/>
-      <c r="H2" s="153" t="s">
+      <c r="G2" s="53"/>
+      <c r="H2" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="149" t="s">
+      <c r="I2" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="149" t="s">
+      <c r="J2" s="67" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="154"/>
-      <c r="I3" s="150"/>
-      <c r="J3" s="150"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
@@ -6461,7 +5869,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="6"/>
+      <c r="I4" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -6497,68 +5905,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="157" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="155" t="s">
+      <c r="I1" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="155"/>
+      <c r="J1" s="73"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="106"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="110" t="s">
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="111"/>
-      <c r="F2" s="110" t="s">
+      <c r="E2" s="53"/>
+      <c r="F2" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="111"/>
-      <c r="H2" s="158"/>
-      <c r="I2" s="156"/>
-      <c r="J2" s="156"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="74"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="158"/>
-      <c r="I3" s="7" t="s">
+      <c r="H3" s="76"/>
+      <c r="I3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="6" t="s">
         <v>31</v>
       </c>
     </row>
@@ -6593,736 +6001,736 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="15"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="17"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="15"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="G4" s="18"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="20"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="18"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" s="15" t="s">
+      <c r="D5" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="17"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="15"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="15" t="s">
+      <c r="D6" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F6" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G6" s="18"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="20"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="18"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="15" t="s">
+      <c r="D7" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G7" s="18"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="20"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="18"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F8" s="15" t="s">
+      <c r="D8" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F8" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="18"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="20"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="18"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F9" s="15" t="s">
+      <c r="D9" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F9" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G9" s="18"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="20"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="18"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F10" s="15" t="s">
+      <c r="D10" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F10" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G10" s="18"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="20"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="18"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F11" s="15" t="s">
+      <c r="D11" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F11" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="18"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="20"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="18"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F12" s="15" t="s">
+      <c r="D12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G12" s="18"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="20"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="18"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F13" s="15" t="s">
+      <c r="D13" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="20"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="18"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F14" s="15" t="s">
+      <c r="D14" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G14" s="18"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="20"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="18"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="15" t="s">
+      <c r="D15" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="18"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="20"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="18"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="D16" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F16" s="15" t="s">
+      <c r="D16" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G16" s="18"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="20"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="D17" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="15" t="s">
+      <c r="D17" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G17" s="18"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="20"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="18"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E18" s="15" t="s">
+      <c r="D18" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G18" s="18"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="20"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="18"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E19" s="15" t="s">
+      <c r="D19" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E19" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="20"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="18"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="D20" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E20" s="15" t="s">
+      <c r="D20" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="20"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="18"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D21" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" s="15" t="s">
+      <c r="D21" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E21" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="F21" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="18"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="20"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="18"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D22" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="15" t="s">
+      <c r="D22" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E22" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G22" s="18"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="20"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="18"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G23" s="18"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="20"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="18"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="D24" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E24" s="15" t="s">
+      <c r="D24" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E24" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="20"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="18"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="F25" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="20"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="18"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="E26" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="F26" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G26" s="18"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="20"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="18"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D27" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E27" s="15" t="s">
+      <c r="D27" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="F27" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G27" s="18"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="20"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="18"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D28" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F28" s="15" t="s">
+      <c r="D28" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F28" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="G28" s="18"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="20"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="18"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="D29" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E29" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F29" s="15" t="s">
+      <c r="D29" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F29" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G29" s="18"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="20"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="18"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="D30" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="F30" s="15" t="s">
+      <c r="D30" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G30" s="18"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="20"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="18"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="22"/>
-      <c r="I31" s="22"/>
-      <c r="J31" s="22"/>
-      <c r="K31" s="22"/>
-      <c r="L31" s="23"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7340,623 +6748,623 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="11" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14">
+      <c r="A2" s="12">
         <v>1688</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" s="14" t="s">
+      <c r="E2" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14">
+      <c r="A3" s="12">
         <v>1691</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F3" s="14" t="s">
+      <c r="E3" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
+      <c r="A4" s="12">
         <v>3980</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G4" s="14" t="s">
+      <c r="E4" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="12">
         <v>5102</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="E5" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F5" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
+      <c r="A6" s="12">
         <v>9930</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="12">
         <v>30645168794</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6" s="14" t="s">
+      <c r="E6" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
+      <c r="A7" s="12">
         <v>12112</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="12">
         <v>30571865684</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="14" t="s">
+      <c r="E7" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14">
+      <c r="A8" s="12">
         <v>12188</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="E8" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G8" s="14" t="s">
+      <c r="E8" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G8" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14">
+      <c r="A9" s="12">
         <v>12700</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E9" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F9" s="14" t="s">
+      <c r="E9" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F9" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14">
+      <c r="A10" s="12">
         <v>13239</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="12">
         <v>30630467620</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14">
+      <c r="A11" s="12">
         <v>24441</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="E11" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F11" s="14" t="s">
+      <c r="E11" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F11" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14">
+      <c r="A12" s="12">
         <v>48440</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="14">
+      <c r="A13" s="12">
         <v>69790</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="12">
         <v>33689822989</v>
       </c>
-      <c r="E13" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G13" s="14" t="s">
+      <c r="E13" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14">
+      <c r="A14" s="12">
         <v>92132</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="12">
         <v>30686692899</v>
       </c>
-      <c r="E14" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G14" s="14" t="s">
+      <c r="E14" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14">
+      <c r="A15" s="12">
         <v>125649</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="E15" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G15" s="14" t="s">
+      <c r="E15" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14">
+      <c r="A16" s="12">
         <v>153200</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="12">
         <v>30707421041</v>
       </c>
-      <c r="E16" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G16" s="14" t="s">
+      <c r="E16" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G16" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14">
+      <c r="A17" s="12">
         <v>167215</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="12">
         <v>30707919902</v>
       </c>
-      <c r="E17" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G17" s="14" t="s">
+      <c r="E17" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14">
+      <c r="A18" s="12">
         <v>173985</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="12">
         <v>30672616774</v>
       </c>
-      <c r="E18" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F18" s="14" t="s">
+      <c r="E18" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G18" s="14" t="s">
+      <c r="G18" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14">
+      <c r="A19" s="12">
         <v>196990</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="12">
         <v>30708617888</v>
       </c>
-      <c r="E19" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G19" s="14" t="s">
+      <c r="E19" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14">
+      <c r="A20" s="12">
         <v>250244</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="E20" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G20" s="14" t="s">
+      <c r="E20" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G20" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14">
+      <c r="A21" s="12">
         <v>250552</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="E21" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G21" s="14" t="s">
+      <c r="E21" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
+      <c r="A22" s="12">
         <v>316725</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="E22" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G22" s="14" t="s">
+      <c r="E22" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14">
+      <c r="A23" s="12">
         <v>344829</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="E23" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G23" s="14" t="s">
+      <c r="E23" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G23" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
+      <c r="A24" s="12">
         <v>374869</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="12">
         <v>30711273197</v>
       </c>
-      <c r="E24" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G24" s="14" t="s">
+      <c r="E24" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G24" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="14">
+      <c r="A25" s="12">
         <v>384417</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="12">
         <v>30711513562</v>
       </c>
-      <c r="E25" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G25" s="14" t="s">
+      <c r="E25" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G25" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="14">
+      <c r="A26" s="12">
         <v>490353</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G26" s="14" t="s">
+      <c r="G26" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="14">
+      <c r="A27" s="12">
         <v>594725</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="14">
+      <c r="D27" s="12">
         <v>30715273906</v>
       </c>
-      <c r="E27" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G27" s="14" t="s">
+      <c r="E27" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" s="12" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
--FIX DE BUG EN EL ARMADO DE LOTES DONDE EL NUMERO DE FACTURA INICIAL DEL LOTE NO SE ACTUALIZABA CORRECTAMENTE
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/PLANTILLA.xlsx
+++ b/Control de Facturas/Assets/Plantillas/PLANTILLA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B5FF04-54EC-42EE-80D0-2A3B94EDDA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F78A279-7C8D-4287-BDDC-AB7BD5E82A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-60" windowWidth="20730" windowHeight="11040" tabRatio="900" xr2:uid="{D9D33F21-ED07-47A1-8533-367C0DEB1D0B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="900" activeTab="3" xr2:uid="{D9D33F21-ED07-47A1-8533-367C0DEB1D0B}"/>
   </bookViews>
   <sheets>
     <sheet name="Cabecera-Cpte" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="10" r:id="rId9"/>
+    <pivotCache cacheId="0" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -2060,7 +2060,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="158">
   <si>
     <t>Observaciones</t>
   </si>
@@ -2531,12 +2531,6 @@
   </si>
   <si>
     <t>Total general</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>COD</t>
   </si>
   <si>
     <t>3.1.1-2390-1</t>
@@ -3480,10 +3474,10 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3628,20 +3622,7 @@
     <cellStyle name="Título 3" xfId="40" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="41" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -3997,7 +3978,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FB68EB4-76D3-458C-A6F3-4728B0F719D5}" name="Tabla dinámica2" cacheId="10" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FB68EB4-76D3-458C-A6F3-4728B0F719D5}" name="Tabla dinámica2" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
   <location ref="A3:L31" firstHeaderRow="2" firstDataRow="2" firstDataCol="6"/>
   <pivotFields count="7">
     <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
@@ -4608,7 +4589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2EE6AC-AB02-466B-BB1F-3973D9012F54}">
-  <dimension ref="A1:AM5"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" style="28" bestFit="1" customWidth="1"/>
@@ -4647,151 +4628,147 @@
     <col min="34" max="34" width="9.42578125" style="29" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="16.5703125" style="42" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="37.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="5" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="3.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="20.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="15.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="7.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="15.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="7.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="18.140625" style="29" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
     <col min="50" max="50" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="22.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="3.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="3.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="7" style="29" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="4.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="6.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="23" style="29" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="14" style="29" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="22.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="4" style="29" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="3.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="3.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="7" style="29" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="4.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="6.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="23" style="29" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="14" style="29" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="12.140625" style="29" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
     <col min="73" max="73" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="79" max="80" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="23.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="25.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="35.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="16.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="23.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="25.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="34.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="16.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="14.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="133" max="135" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="136" max="16384" width="11.42578125" style="29"/>
+    <col min="74" max="74" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="75" max="76" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="23.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="25.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="35.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="16.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="12.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="23.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="25.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="34.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="16.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="14.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
+    <col min="129" max="131" width="13.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="132" max="16384" width="11.42578125" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A1" s="44" t="s">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A1" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="44"/>
-      <c r="AB1" s="44"/>
-      <c r="AC1" s="44"/>
-      <c r="AD1" s="44"/>
-      <c r="AE1" s="44"/>
-      <c r="AF1" s="44"/>
-      <c r="AG1" s="44"/>
-      <c r="AH1" s="44"/>
-      <c r="AI1" s="44"/>
-      <c r="AJ1" s="44"/>
-    </row>
-    <row r="2" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A2" s="43" t="s">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
+      <c r="AA1" s="43"/>
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
+      <c r="AD1" s="43"/>
+      <c r="AE1" s="43"/>
+      <c r="AF1" s="43"/>
+      <c r="AG1" s="43"/>
+      <c r="AH1" s="43"/>
+      <c r="AI1" s="43"/>
+      <c r="AJ1" s="43"/>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A2" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="45" t="s">
         <v>78</v>
       </c>
@@ -4809,96 +4786,96 @@
         <v>11</v>
       </c>
       <c r="P2" s="45"/>
-      <c r="Q2" s="43" t="s">
+      <c r="Q2" s="44" t="s">
         <v>67</v>
       </c>
-      <c r="R2" s="43"/>
-      <c r="S2" s="43"/>
-      <c r="T2" s="43"/>
-      <c r="U2" s="43" t="s">
+      <c r="R2" s="44"/>
+      <c r="S2" s="44"/>
+      <c r="T2" s="44"/>
+      <c r="U2" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="V2" s="43"/>
-      <c r="W2" s="43"/>
-      <c r="X2" s="43" t="s">
+      <c r="V2" s="44"/>
+      <c r="W2" s="44"/>
+      <c r="X2" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="Y2" s="43"/>
-      <c r="Z2" s="43"/>
-      <c r="AA2" s="43"/>
-      <c r="AB2" s="43" t="s">
+      <c r="Y2" s="44"/>
+      <c r="Z2" s="44"/>
+      <c r="AA2" s="44"/>
+      <c r="AB2" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="AC2" s="43" t="s">
+      <c r="AC2" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="AD2" s="43"/>
-      <c r="AE2" s="43"/>
-      <c r="AF2" s="43" t="s">
+      <c r="AD2" s="44"/>
+      <c r="AE2" s="44"/>
+      <c r="AF2" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="AG2" s="43"/>
-      <c r="AH2" s="43"/>
+      <c r="AG2" s="44"/>
+      <c r="AH2" s="44"/>
       <c r="AI2" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="AJ2" s="43" t="s">
+      <c r="AJ2" s="44" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:39" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="43"/>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43" t="s">
+    <row r="3" spans="1:36" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="43" t="s">
+      <c r="E3" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
       <c r="H3" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="43" t="s">
+      <c r="I3" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="J3" s="43"/>
+      <c r="J3" s="44"/>
       <c r="K3" s="32" t="s">
         <v>84</v>
       </c>
       <c r="L3" s="27"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="43" t="s">
+      <c r="N3" s="44" t="s">
         <v>80</v>
       </c>
       <c r="O3" s="45" t="s">
         <v>34</v>
       </c>
       <c r="P3" s="45"/>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="43"/>
-      <c r="S3" s="43"/>
-      <c r="T3" s="43"/>
-      <c r="U3" s="43"/>
-      <c r="V3" s="43"/>
-      <c r="W3" s="43"/>
-      <c r="X3" s="43"/>
-      <c r="Y3" s="43"/>
-      <c r="Z3" s="43"/>
-      <c r="AA3" s="43"/>
-      <c r="AB3" s="43"/>
-      <c r="AC3" s="43"/>
-      <c r="AD3" s="43"/>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="43"/>
-      <c r="AG3" s="43"/>
-      <c r="AH3" s="43"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="44"/>
+      <c r="U3" s="44"/>
+      <c r="V3" s="44"/>
+      <c r="W3" s="44"/>
+      <c r="X3" s="44"/>
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="44"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="44"/>
+      <c r="AD3" s="44"/>
+      <c r="AE3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="44"/>
+      <c r="AH3" s="44"/>
       <c r="AI3" s="46"/>
-      <c r="AJ3" s="43"/>
-    </row>
-    <row r="4" spans="1:39" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AJ3" s="44"/>
+    </row>
+    <row r="4" spans="1:36" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
         <v>39</v>
       </c>
@@ -4908,7 +4885,7 @@
       <c r="C4" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="43"/>
+      <c r="D4" s="44"/>
       <c r="E4" s="29" t="s">
         <v>35</v>
       </c>
@@ -4936,7 +4913,7 @@
       <c r="M4" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="N4" s="43"/>
+      <c r="N4" s="44"/>
       <c r="O4" s="30" t="s">
         <v>13</v>
       </c>
@@ -4976,7 +4953,7 @@
       <c r="AA4" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="AB4" s="43"/>
+      <c r="AB4" s="44"/>
       <c r="AC4" s="30" t="s">
         <v>13</v>
       </c>
@@ -4998,18 +4975,9 @@
       <c r="AI4" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="AJ4" s="43"/>
-      <c r="AK4" s="29" t="s">
-        <v>158</v>
-      </c>
-      <c r="AL4" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="AM4" s="29" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:39" x14ac:dyDescent="0.2">
+      <c r="AJ4" s="44"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="28">
         <v>326</v>
       </c>
@@ -5050,13 +5018,10 @@
       <c r="AH5" s="30"/>
       <c r="AI5" s="40"/>
       <c r="AJ5" s="30"/>
-      <c r="AM5" s="29">
-        <f>LEN(AJ5)</f>
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="N3:N4"/>
     <mergeCell ref="A1:AJ1"/>
     <mergeCell ref="A2:C3"/>
     <mergeCell ref="O2:P2"/>
@@ -5073,14 +5038,8 @@
     <mergeCell ref="X2:AA3"/>
     <mergeCell ref="U2:W3"/>
     <mergeCell ref="E3:G3"/>
-    <mergeCell ref="N3:N4"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="AM1:AM1048576">
-    <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="greaterThan">
-      <formula>255</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" blackAndWhite="1" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -5353,7 +5312,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="29" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J4" s="29">
         <v>3</v>
@@ -5447,37 +5406,37 @@
       <c r="E1" s="45"/>
       <c r="F1" s="45"/>
       <c r="G1" s="45"/>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="44"/>
-      <c r="AB1" s="44"/>
-      <c r="AC1" s="44"/>
-      <c r="AD1" s="44"/>
-      <c r="AE1" s="44"/>
-      <c r="AF1" s="44"/>
-      <c r="AG1" s="44"/>
-      <c r="AH1" s="44"/>
-      <c r="AI1" s="44"/>
-      <c r="AJ1" s="44"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
+      <c r="AA1" s="43"/>
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
+      <c r="AD1" s="43"/>
+      <c r="AE1" s="43"/>
+      <c r="AF1" s="43"/>
+      <c r="AG1" s="43"/>
+      <c r="AH1" s="43"/>
+      <c r="AI1" s="43"/>
+      <c r="AJ1" s="43"/>
     </row>
     <row r="2" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="45" t="s">
@@ -5499,33 +5458,33 @@
       <c r="I2" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="J2" s="43" t="s">
+      <c r="J2" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43" t="s">
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="N2" s="43" t="s">
+      <c r="N2" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="43" t="s">
+      <c r="O2" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="P2" s="43"/>
-      <c r="Q2" s="43"/>
-      <c r="R2" s="43"/>
-      <c r="S2" s="43"/>
-      <c r="T2" s="43" t="s">
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
+      <c r="S2" s="44"/>
+      <c r="T2" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="43" t="s">
+      <c r="U2" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="V2" s="43"/>
-      <c r="W2" s="43"/>
-      <c r="X2" s="43"/>
+      <c r="V2" s="44"/>
+      <c r="W2" s="44"/>
+      <c r="X2" s="44"/>
       <c r="Y2" s="45" t="s">
         <v>61</v>
       </c>
@@ -5596,8 +5555,8 @@
       <c r="L3" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
       <c r="O3" s="29" t="s">
         <v>52</v>
       </c>
@@ -5613,7 +5572,7 @@
       <c r="S3" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="T3" s="43"/>
+      <c r="T3" s="44"/>
       <c r="U3" s="29" t="s">
         <v>57</v>
       </c>
@@ -5743,6 +5702,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="AH2:AH3"/>
+    <mergeCell ref="O2:S2"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="U2:X2"/>
     <mergeCell ref="H1:AJ1"/>
     <mergeCell ref="Y2:Y3"/>
     <mergeCell ref="Z2:Z3"/>
@@ -5759,15 +5727,6 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="N2:N3"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="AH2:AH3"/>
-    <mergeCell ref="O2:S2"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="U2:X2"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
--IMPLEMENTACION DE CONVERSOR DE XLSX A XLS, PARA LA CORRECTA IMPORTACION AL SISTEMA SIDIF
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/PLANTILLA.xlsx
+++ b/Control de Facturas/Assets/Plantillas/PLANTILLA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F78A279-7C8D-4287-BDDC-AB7BD5E82A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C7465C-4312-4449-8C2A-1D9CD370B27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="900" activeTab="3" xr2:uid="{D9D33F21-ED07-47A1-8533-367C0DEB1D0B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="900" xr2:uid="{D9D33F21-ED07-47A1-8533-367C0DEB1D0B}"/>
   </bookViews>
   <sheets>
     <sheet name="Cabecera-Cpte" sheetId="4" r:id="rId1"/>
@@ -19,16 +19,11 @@
     <sheet name="Detalle Presupuestario  FACGS" sheetId="8" r:id="rId4"/>
     <sheet name="Deducciones" sheetId="9" r:id="rId5"/>
     <sheet name="Det Deducc x Cptos" sheetId="13" r:id="rId6"/>
-    <sheet name="Hoja4" sheetId="18" r:id="rId7"/>
-    <sheet name="BENEFICIARIOS" sheetId="17" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pronto Pago'!$A$2:$C$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId9"/>
-  </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2060,7 +2055,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="96">
   <si>
     <t>Observaciones</t>
   </si>
@@ -2335,9 +2330,6 @@
     <t>B</t>
   </si>
   <si>
-    <t>CESP</t>
-  </si>
-  <si>
     <t>CUI</t>
   </si>
   <si>
@@ -2348,189 +2340,6 @@
   </si>
   <si>
     <t>RC</t>
-  </si>
-  <si>
-    <t>Denominación</t>
-  </si>
-  <si>
-    <t>CUIT</t>
-  </si>
-  <si>
-    <t>GAN</t>
-  </si>
-  <si>
-    <t>N/A Cod. Autorización</t>
-  </si>
-  <si>
-    <t>ENTE PROVINCIAL DE AGUA Y SANEAMIENTO</t>
-  </si>
-  <si>
-    <t>30999273498</t>
-  </si>
-  <si>
-    <t>RI</t>
-  </si>
-  <si>
-    <t>D.P.O.S.S. DIRECCION PROVINCIAL DE OBRAS Y SERVICIOS SANITARIOS</t>
-  </si>
-  <si>
-    <t>30587083074</t>
-  </si>
-  <si>
-    <t>NI</t>
-  </si>
-  <si>
-    <t>SERVICIO DE AGUA Y MANTENIMIENTO EMPRESA DEL ESTADO PROVINCIAL S A M E E P</t>
-  </si>
-  <si>
-    <t>30556366906</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>OBRAS SANITARIAS SOCIEDAD DEL ESTADO SAN JUAN</t>
-  </si>
-  <si>
-    <t>30999032849</t>
-  </si>
-  <si>
-    <t>AGUAS DE CORRIENTES S.A.</t>
-  </si>
-  <si>
-    <t>30645168794</t>
-  </si>
-  <si>
-    <t>COOPERATIVA DE AGUA POTABLE Y OTROS SERVICIOS PUB DE SAN MARTIN DE LOS ANDES</t>
-  </si>
-  <si>
-    <t>30571865684</t>
-  </si>
-  <si>
-    <t>AGUAS DE FORMOSA SA.</t>
-  </si>
-  <si>
-    <t>30671378047</t>
-  </si>
-  <si>
-    <t>COOPERATIVA DE TRABAJO 15 DE MAYO LIMITADA</t>
-  </si>
-  <si>
-    <t>30651082575</t>
-  </si>
-  <si>
-    <t>OBRAS SANITARIAS DE MAR DEL PLATA S.E.</t>
-  </si>
-  <si>
-    <t>30630467620</t>
-  </si>
-  <si>
-    <t>NC</t>
-  </si>
-  <si>
-    <t>COOPERATIVA DE TRABAJO SUDESTE LTDA.</t>
-  </si>
-  <si>
-    <t>30668249651</t>
-  </si>
-  <si>
-    <t>OBRAS SANITARIAS MUNICIPAL - ENTE DESCENTRALIZADO</t>
-  </si>
-  <si>
-    <t>30642668281</t>
-  </si>
-  <si>
-    <t>AGUAS CORDOBESAS S.A.</t>
-  </si>
-  <si>
-    <t>33689822989</t>
-  </si>
-  <si>
-    <t>AGUAS DE SANTIAGO S.A.</t>
-  </si>
-  <si>
-    <t>30686692899</t>
-  </si>
-  <si>
-    <t>SERVICIOS DE AGUA DE MISIONES S A</t>
-  </si>
-  <si>
-    <t>33698095909</t>
-  </si>
-  <si>
-    <t>AGUAS RIONEGRINAS SOCIEDAD ANONIMA</t>
-  </si>
-  <si>
-    <t>30707421041</t>
-  </si>
-  <si>
-    <t>AGUAS BONAERENSES S.A.</t>
-  </si>
-  <si>
-    <t>30707919902</t>
-  </si>
-  <si>
-    <t>ENTE AUTARQUICO MUNICIPAL DE SERVICIO PUBLICOS (EAMSEP)</t>
-  </si>
-  <si>
-    <t>30672616774</t>
-  </si>
-  <si>
-    <t>SOCIEDAD DE AGUAS DEL TUCUMAN - SAPEM</t>
-  </si>
-  <si>
-    <t>30708617888</t>
-  </si>
-  <si>
-    <t>AGUA Y SANEAMIENTOS ARGENTINOS S.A.</t>
-  </si>
-  <si>
-    <t>30709565075</t>
-  </si>
-  <si>
-    <t>AGUAS SANTAFESINAS  S.A.</t>
-  </si>
-  <si>
-    <t>30709514144</t>
-  </si>
-  <si>
-    <t>AGUAS DE CATAMARCA S.A. CON PARTICIPACION ESTATAL MAYORITARIA S.A.P.E.M.</t>
-  </si>
-  <si>
-    <t>30710500513</t>
-  </si>
-  <si>
-    <t>COMPAÑIA SALTEÑA DE AGUA Y SANEAMIENTO S.A</t>
-  </si>
-  <si>
-    <t>33710974549</t>
-  </si>
-  <si>
-    <t>AGUAS RIOJANAS S.A.P.E.M.</t>
-  </si>
-  <si>
-    <t>30711273197</t>
-  </si>
-  <si>
-    <t>AGUA Y SANEAMIENTO MENDOZA S.A.</t>
-  </si>
-  <si>
-    <t>30711513562</t>
-  </si>
-  <si>
-    <t>ENTE MUNICIPAL DE OBRAS Y SERVICIOS DE SANEAMIENTO  E M O S S</t>
-  </si>
-  <si>
-    <t>30668543339</t>
-  </si>
-  <si>
-    <t>AGUA POTABLE Y SANEAMIENTO DE JUJUY SOCIEDAD DEL ESTADO</t>
-  </si>
-  <si>
-    <t>30715273906</t>
-  </si>
-  <si>
-    <t>Total general</t>
   </si>
   <si>
     <t>3.1.1-2390-1</t>
@@ -2544,7 +2353,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_ [$€-2]\ * #,##0.00_ ;_ [$€-2]\ * \-#,##0.00_ ;_ [$€-2]\ * &quot;-&quot;??_ "/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2736,20 +2545,13 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="30">
+  <fills count="29">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2896,14 +2698,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="36">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -3082,158 +2878,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="8"/>
-      </left>
-      <right style="medium">
-        <color indexed="8"/>
-      </right>
-      <top style="medium">
-        <color indexed="8"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -3376,7 +3020,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3402,24 +3046,6 @@
     <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" pivotButton="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="2" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3447,25 +3073,25 @@
     <xf numFmtId="0" fontId="2" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="31" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="14" fontId="32" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="31" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="44" fontId="32" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="31" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3474,25 +3100,28 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3510,7 +3139,7 @@
     <xf numFmtId="49" fontId="0" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="27" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="27" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3519,13 +3148,13 @@
     <xf numFmtId="0" fontId="2" fillId="27" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="27" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3540,28 +3169,25 @@
     <xf numFmtId="0" fontId="2" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="28" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3570,7 +3196,7 @@
     <xf numFmtId="0" fontId="3" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -3633,673 +3259,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Operaor" refreshedDate="45068.590425925926" createdVersion="1" refreshedVersion="3" recordCount="26" upgradeOnRefresh="1" xr:uid="{4531BB3F-135A-4B3F-A60C-3BBD24AE6D0A}">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A1:G27" sheet="BENEFICIARIOS"/>
-  </cacheSource>
-  <cacheFields count="7">
-    <cacheField name="Número" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1688" maxValue="594725"/>
-    </cacheField>
-    <cacheField name="Denominación" numFmtId="0">
-      <sharedItems count="26">
-        <s v="ENTE PROVINCIAL DE AGUA Y SANEAMIENTO"/>
-        <s v="D.P.O.S.S. DIRECCION PROVINCIAL DE OBRAS Y SERVICIOS SANITARIOS"/>
-        <s v="SERVICIO DE AGUA Y MANTENIMIENTO EMPRESA DEL ESTADO PROVINCIAL S A M E E P"/>
-        <s v="OBRAS SANITARIAS SOCIEDAD DEL ESTADO SAN JUAN"/>
-        <s v="AGUAS DE CORRIENTES S.A."/>
-        <s v="COOPERATIVA DE AGUA POTABLE Y OTROS SERVICIOS PUB DE SAN MARTIN DE LOS ANDES"/>
-        <s v="AGUAS DE FORMOSA SA."/>
-        <s v="COOPERATIVA DE TRABAJO 15 DE MAYO LIMITADA"/>
-        <s v="OBRAS SANITARIAS DE MAR DEL PLATA S.E."/>
-        <s v="COOPERATIVA DE TRABAJO SUDESTE LTDA."/>
-        <s v="OBRAS SANITARIAS MUNICIPAL - ENTE DESCENTRALIZADO"/>
-        <s v="AGUAS CORDOBESAS S.A."/>
-        <s v="AGUAS DE SANTIAGO S.A."/>
-        <s v="SERVICIOS DE AGUA DE MISIONES S A"/>
-        <s v="AGUAS RIONEGRINAS SOCIEDAD ANONIMA"/>
-        <s v="AGUAS BONAERENSES S.A."/>
-        <s v="ENTE AUTARQUICO MUNICIPAL DE SERVICIO PUBLICOS (EAMSEP)"/>
-        <s v="SOCIEDAD DE AGUAS DEL TUCUMAN - SAPEM"/>
-        <s v="AGUA Y SANEAMIENTOS ARGENTINOS S.A."/>
-        <s v="AGUAS SANTAFESINAS  S.A."/>
-        <s v="AGUAS DE CATAMARCA S.A. CON PARTICIPACION ESTATAL MAYORITARIA S.A.P.E.M."/>
-        <s v="COMPAÑIA SALTEÑA DE AGUA Y SANEAMIENTO S.A"/>
-        <s v="AGUAS RIOJANAS S.A.P.E.M."/>
-        <s v="AGUA Y SANEAMIENTO MENDOZA S.A."/>
-        <s v="ENTE MUNICIPAL DE OBRAS Y SERVICIOS DE SANEAMIENTO  E M O S S"/>
-        <s v="AGUA POTABLE Y SANEAMIENTO DE JUJUY SOCIEDAD DEL ESTADO"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="CUI" numFmtId="0">
-      <sharedItems count="1">
-        <s v="CUI"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="CUIT" numFmtId="0">
-      <sharedItems count="26">
-        <s v="30999273498"/>
-        <s v="30587083074"/>
-        <s v="30556366906"/>
-        <s v="30999032849"/>
-        <s v="30645168794"/>
-        <s v="30571865684"/>
-        <s v="30671378047"/>
-        <s v="30651082575"/>
-        <s v="30630467620"/>
-        <s v="30668249651"/>
-        <s v="30642668281"/>
-        <s v="33689822989"/>
-        <s v="30686692899"/>
-        <s v="33698095909"/>
-        <s v="30707421041"/>
-        <s v="30707919902"/>
-        <s v="30672616774"/>
-        <s v="30708617888"/>
-        <s v="30709565075"/>
-        <s v="30709514144"/>
-        <s v="30710500513"/>
-        <s v="33710974549"/>
-        <s v="30711273197"/>
-        <s v="30711513562"/>
-        <s v="30668543339"/>
-        <s v="30715273906"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="IVA" numFmtId="0">
-      <sharedItems count="3">
-        <s v="RI"/>
-        <s v="NC"/>
-        <s v="EXE"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="GAN" numFmtId="0">
-      <sharedItems count="3">
-        <s v="EXE"/>
-        <s v="NI"/>
-        <s v="RI"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="N/A Cod. Autorización" numFmtId="0">
-      <sharedItems count="2">
-        <s v="CESP"/>
-        <s v="NA"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="26">
-  <r>
-    <n v="1688"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="1691"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="3980"/>
-    <x v="2"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="5102"/>
-    <x v="3"/>
-    <x v="0"/>
-    <x v="3"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="9930"/>
-    <x v="4"/>
-    <x v="0"/>
-    <x v="4"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="12112"/>
-    <x v="5"/>
-    <x v="0"/>
-    <x v="5"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="12188"/>
-    <x v="6"/>
-    <x v="0"/>
-    <x v="6"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="12700"/>
-    <x v="7"/>
-    <x v="0"/>
-    <x v="7"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="13239"/>
-    <x v="8"/>
-    <x v="0"/>
-    <x v="8"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="24441"/>
-    <x v="9"/>
-    <x v="0"/>
-    <x v="9"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="48440"/>
-    <x v="10"/>
-    <x v="0"/>
-    <x v="10"/>
-    <x v="1"/>
-    <x v="0"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="69790"/>
-    <x v="11"/>
-    <x v="0"/>
-    <x v="11"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="92132"/>
-    <x v="12"/>
-    <x v="0"/>
-    <x v="12"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="125649"/>
-    <x v="13"/>
-    <x v="0"/>
-    <x v="13"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="153200"/>
-    <x v="14"/>
-    <x v="0"/>
-    <x v="14"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="167215"/>
-    <x v="15"/>
-    <x v="0"/>
-    <x v="15"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="173985"/>
-    <x v="16"/>
-    <x v="0"/>
-    <x v="16"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="196990"/>
-    <x v="17"/>
-    <x v="0"/>
-    <x v="17"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="250244"/>
-    <x v="18"/>
-    <x v="0"/>
-    <x v="18"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="250552"/>
-    <x v="19"/>
-    <x v="0"/>
-    <x v="19"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="316725"/>
-    <x v="20"/>
-    <x v="0"/>
-    <x v="20"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="344829"/>
-    <x v="21"/>
-    <x v="0"/>
-    <x v="21"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="374869"/>
-    <x v="22"/>
-    <x v="0"/>
-    <x v="22"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <n v="384417"/>
-    <x v="23"/>
-    <x v="0"/>
-    <x v="23"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="490353"/>
-    <x v="24"/>
-    <x v="0"/>
-    <x v="24"/>
-    <x v="2"/>
-    <x v="0"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <n v="594725"/>
-    <x v="25"/>
-    <x v="0"/>
-    <x v="25"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="0"/>
-  </r>
-</pivotCacheRecords>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FB68EB4-76D3-458C-A6F3-4728B0F719D5}" name="Tabla dinámica2" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
-  <location ref="A3:L31" firstHeaderRow="2" firstDataRow="2" firstDataCol="6"/>
-  <pivotFields count="7">
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1" defaultSubtotal="0">
-      <items count="26">
-        <item x="25"/>
-        <item x="23"/>
-        <item x="18"/>
-        <item x="15"/>
-        <item x="11"/>
-        <item x="20"/>
-        <item x="4"/>
-        <item x="6"/>
-        <item x="12"/>
-        <item x="22"/>
-        <item x="14"/>
-        <item x="19"/>
-        <item x="21"/>
-        <item x="5"/>
-        <item x="7"/>
-        <item x="9"/>
-        <item x="1"/>
-        <item x="16"/>
-        <item x="24"/>
-        <item x="0"/>
-        <item x="8"/>
-        <item x="10"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="13"/>
-        <item x="17"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1" defaultSubtotal="0">
-      <items count="1">
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1" defaultSubtotal="0">
-      <items count="26">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item x="8"/>
-        <item x="10"/>
-        <item x="4"/>
-        <item x="7"/>
-        <item x="9"/>
-        <item x="24"/>
-        <item x="6"/>
-        <item x="16"/>
-        <item x="12"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="17"/>
-        <item x="19"/>
-        <item x="18"/>
-        <item x="20"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="25"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="13"/>
-        <item x="21"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1" defaultSubtotal="0">
-      <items count="3">
-        <item x="2"/>
-        <item x="1"/>
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1" defaultSubtotal="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="6">
-    <field x="1"/>
-    <field x="2"/>
-    <field x="3"/>
-    <field x="4"/>
-    <field x="5"/>
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="27">
-    <i>
-      <x/>
-      <x/>
-      <x v="20"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x/>
-      <x v="19"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x/>
-      <x v="16"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="3"/>
-      <x/>
-      <x v="13"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="4"/>
-      <x/>
-      <x v="23"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="5"/>
-      <x/>
-      <x v="17"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="6"/>
-      <x/>
-      <x v="5"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="7"/>
-      <x/>
-      <x v="9"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="8"/>
-      <x/>
-      <x v="11"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="9"/>
-      <x/>
-      <x v="18"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="10"/>
-      <x/>
-      <x v="12"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="11"/>
-      <x/>
-      <x v="15"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="12"/>
-      <x/>
-      <x v="25"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="13"/>
-      <x/>
-      <x v="1"/>
-      <x v="2"/>
-      <x/>
-      <x/>
-    </i>
-    <i>
-      <x v="14"/>
-      <x/>
-      <x v="6"/>
-      <x v="2"/>
-      <x/>
-      <x/>
-    </i>
-    <i>
-      <x v="15"/>
-      <x/>
-      <x v="7"/>
-      <x v="2"/>
-      <x/>
-      <x/>
-    </i>
-    <i>
-      <x v="16"/>
-      <x/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-      <x/>
-    </i>
-    <i>
-      <x v="17"/>
-      <x/>
-      <x v="10"/>
-      <x v="2"/>
-      <x/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="18"/>
-      <x/>
-      <x v="8"/>
-      <x/>
-      <x/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="19"/>
-      <x/>
-      <x v="22"/>
-      <x v="2"/>
-      <x/>
-      <x/>
-    </i>
-    <i>
-      <x v="20"/>
-      <x/>
-      <x v="3"/>
-      <x v="1"/>
-      <x/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="21"/>
-      <x/>
-      <x v="4"/>
-      <x v="1"/>
-      <x/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="22"/>
-      <x/>
-      <x v="21"/>
-      <x v="2"/>
-      <x v="1"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="23"/>
-      <x/>
-      <x/>
-      <x v="2"/>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="24"/>
-      <x/>
-      <x v="24"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i>
-      <x v="25"/>
-      <x/>
-      <x v="14"/>
-      <x v="2"/>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4592,435 +3551,436 @@
   <dimension ref="A1:AJ5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" style="28" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" style="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" style="36" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" style="36" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" style="36" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.140625" style="28" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="28" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" style="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" style="28" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="5.85546875" style="36" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="7.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12" style="36" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.28515625" style="36" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="16.5703125" style="42" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="37.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="7.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="18.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="22.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="3.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="3.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="7" style="29" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="4.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="6.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="23" style="29" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="14" style="29" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="30.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="75" max="76" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="23.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="25.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="35.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="16.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="13.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="12.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="18.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="10.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="23.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="25.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="34.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="17.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="16.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="15.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="16.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="14.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="2.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="13.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="15.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="9.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="11.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="129" max="131" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="132" max="16384" width="11.42578125" style="29"/>
+    <col min="1" max="1" width="14" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" style="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" style="22" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.28515625" style="22" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" style="27" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4" style="15" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="4.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="7.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12" style="22" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.28515625" style="22" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="16.5703125" style="28" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="37.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="7.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="7.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="5.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="18.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="10.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="22.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="4" style="15" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="4.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="3.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="3.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="7" style="15" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="4.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="2.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="8.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="4.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="4.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="6.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="5.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="23" style="15" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="14" style="15" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="30.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="12.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="18.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="75" max="76" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="23.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="25.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="17.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="17.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="15.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="35.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="17.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="17.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="16.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="15.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="16.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="6.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="2.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="13.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="15.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="9.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="13.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="12.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="18.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="12.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="10.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="23.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="25.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="17.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="17.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="15.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="34.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="17.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="17.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="16.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="15.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="16.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="14.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="6.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="2.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="13.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="15.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="9.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="129" max="131" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="132" max="16384" width="11.42578125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
-      <c r="Z1" s="43"/>
-      <c r="AA1" s="43"/>
-      <c r="AB1" s="43"/>
-      <c r="AC1" s="43"/>
-      <c r="AD1" s="43"/>
-      <c r="AE1" s="43"/>
-      <c r="AF1" s="43"/>
-      <c r="AG1" s="43"/>
-      <c r="AH1" s="43"/>
-      <c r="AI1" s="43"/>
-      <c r="AJ1" s="43"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="31"/>
+      <c r="Y1" s="31"/>
+      <c r="Z1" s="31"/>
+      <c r="AA1" s="31"/>
+      <c r="AB1" s="31"/>
+      <c r="AC1" s="31"/>
+      <c r="AD1" s="31"/>
+      <c r="AE1" s="31"/>
+      <c r="AF1" s="31"/>
+      <c r="AG1" s="31"/>
+      <c r="AH1" s="31"/>
+      <c r="AI1" s="31"/>
+      <c r="AJ1" s="31"/>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="45" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45" t="s">
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="44" t="s">
+      <c r="P2" s="29"/>
+      <c r="Q2" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
-      <c r="T2" s="44"/>
-      <c r="U2" s="44" t="s">
+      <c r="R2" s="30"/>
+      <c r="S2" s="30"/>
+      <c r="T2" s="30"/>
+      <c r="U2" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="V2" s="44"/>
-      <c r="W2" s="44"/>
-      <c r="X2" s="44" t="s">
+      <c r="V2" s="30"/>
+      <c r="W2" s="30"/>
+      <c r="X2" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="Y2" s="44"/>
-      <c r="Z2" s="44"/>
-      <c r="AA2" s="44"/>
-      <c r="AB2" s="44" t="s">
+      <c r="Y2" s="30"/>
+      <c r="Z2" s="30"/>
+      <c r="AA2" s="30"/>
+      <c r="AB2" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="AC2" s="44" t="s">
+      <c r="AC2" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="AD2" s="44"/>
-      <c r="AE2" s="44"/>
-      <c r="AF2" s="44" t="s">
+      <c r="AD2" s="30"/>
+      <c r="AE2" s="30"/>
+      <c r="AF2" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="AG2" s="44"/>
-      <c r="AH2" s="44"/>
-      <c r="AI2" s="46" t="s">
+      <c r="AG2" s="30"/>
+      <c r="AH2" s="30"/>
+      <c r="AI2" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="AJ2" s="44" t="s">
+      <c r="AJ2" s="30" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:36" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="44"/>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44" t="s">
+      <c r="A3" s="30"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="44" t="s">
+      <c r="E3" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="32" t="s">
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="44" t="s">
+      <c r="I3" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="J3" s="44"/>
-      <c r="K3" s="32" t="s">
+      <c r="J3" s="30"/>
+      <c r="K3" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="L3" s="27"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="44" t="s">
+      <c r="L3" s="13"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="O3" s="45" t="s">
+      <c r="O3" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="44"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44"/>
-      <c r="T3" s="44"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="44"/>
-      <c r="W3" s="44"/>
-      <c r="X3" s="44"/>
-      <c r="Y3" s="44"/>
-      <c r="Z3" s="44"/>
-      <c r="AA3" s="44"/>
-      <c r="AB3" s="44"/>
-      <c r="AC3" s="44"/>
-      <c r="AD3" s="44"/>
-      <c r="AE3" s="44"/>
-      <c r="AF3" s="44"/>
-      <c r="AG3" s="44"/>
-      <c r="AH3" s="44"/>
-      <c r="AI3" s="46"/>
-      <c r="AJ3" s="44"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="30"/>
+      <c r="R3" s="30"/>
+      <c r="S3" s="30"/>
+      <c r="T3" s="30"/>
+      <c r="U3" s="30"/>
+      <c r="V3" s="30"/>
+      <c r="W3" s="30"/>
+      <c r="X3" s="30"/>
+      <c r="Y3" s="30"/>
+      <c r="Z3" s="30"/>
+      <c r="AA3" s="30"/>
+      <c r="AB3" s="30"/>
+      <c r="AC3" s="30"/>
+      <c r="AD3" s="30"/>
+      <c r="AE3" s="30"/>
+      <c r="AF3" s="30"/>
+      <c r="AG3" s="30"/>
+      <c r="AH3" s="30"/>
+      <c r="AI3" s="33"/>
+      <c r="AJ3" s="30"/>
     </row>
     <row r="4" spans="1:36" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="44"/>
-      <c r="E4" s="29" t="s">
+      <c r="D4" s="30"/>
+      <c r="E4" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="G4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="36" t="s">
+      <c r="H4" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="J4" s="36" t="s">
+      <c r="J4" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="K4" s="29" t="s">
+      <c r="K4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="29" t="s">
+      <c r="M4" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="N4" s="44"/>
-      <c r="O4" s="30" t="s">
+      <c r="N4" s="30"/>
+      <c r="O4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="28" t="s">
+      <c r="P4" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="30" t="s">
+      <c r="Q4" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="R4" s="30" t="s">
+      <c r="R4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="S4" s="29" t="s">
+      <c r="S4" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="T4" s="29" t="s">
+      <c r="T4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="U4" s="30" t="s">
+      <c r="U4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="V4" s="30" t="s">
+      <c r="V4" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="W4" s="30" t="s">
+      <c r="W4" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="X4" s="30" t="s">
+      <c r="X4" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="Y4" s="30" t="s">
+      <c r="Y4" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="Z4" s="32" t="s">
+      <c r="Z4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="AA4" s="30" t="s">
+      <c r="AA4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="AB4" s="44"/>
-      <c r="AC4" s="30" t="s">
+      <c r="AB4" s="30"/>
+      <c r="AC4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="AD4" s="30" t="s">
+      <c r="AD4" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="AE4" s="30" t="s">
+      <c r="AE4" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="AF4" s="32" t="s">
+      <c r="AF4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="AG4" s="32" t="s">
+      <c r="AG4" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="AH4" s="30" t="s">
+      <c r="AH4" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="AI4" s="31" t="s">
+      <c r="AI4" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="AJ4" s="44"/>
+      <c r="AJ4" s="30"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A5" s="28">
+      <c r="A5" s="14">
         <v>326</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="15">
         <f ca="1">YEAR(TODAY())</f>
         <v>2026</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="39"/>
-      <c r="O5" s="29" t="s">
-        <v>92</v>
-      </c>
-      <c r="X5" s="29" t="s">
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="25"/>
+      <c r="O5" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="X5" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA5" s="15">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="AA5" s="29">
-        <v>1</v>
-      </c>
-      <c r="AB5" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="AF5" s="38"/>
-      <c r="AG5" s="38"/>
-      <c r="AH5" s="30"/>
-      <c r="AI5" s="40"/>
-      <c r="AJ5" s="30"/>
+      <c r="AF5" s="24"/>
+      <c r="AG5" s="24"/>
+      <c r="AH5" s="16"/>
+      <c r="AI5" s="26"/>
+      <c r="AJ5" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="E3:G3"/>
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="A1:AJ1"/>
     <mergeCell ref="A2:C3"/>
@@ -5037,7 +3997,6 @@
     <mergeCell ref="AB2:AB4"/>
     <mergeCell ref="X2:AA3"/>
     <mergeCell ref="U2:W3"/>
-    <mergeCell ref="E3:G3"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -5064,42 +4023,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="56" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="52" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="53"/>
-      <c r="F2" s="52" t="s">
+      <c r="E2" s="40"/>
+      <c r="F2" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="54" t="s">
+      <c r="G2" s="40"/>
+      <c r="H2" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="57" t="s">
+      <c r="I2" s="44" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="59" t="s">
+      <c r="J2" s="46" t="s">
         <v>0</v>
       </c>
     </row>
@@ -5125,9 +4084,9 @@
       <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="55"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="60"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5153,183 +4112,183 @@
   <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" style="28" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" style="29" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" style="28" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.140625" style="29" customWidth="1"/>
-    <col min="10" max="10" width="5.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" style="29"/>
-    <col min="13" max="13" width="14.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" style="29" customWidth="1"/>
-    <col min="16" max="16" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14" style="29" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="11.42578125" style="29"/>
+    <col min="1" max="1" width="5.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" style="15" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.140625" style="15" customWidth="1"/>
+    <col min="10" max="10" width="5.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" style="15"/>
+    <col min="13" max="13" width="14.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" style="15" customWidth="1"/>
+    <col min="16" max="16" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14" style="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="11.42578125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
-      <c r="P1" s="63"/>
-      <c r="Q1" s="63"/>
-      <c r="R1" s="63"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
     </row>
     <row r="2" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61" t="s">
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61" t="s">
+      <c r="E2" s="48"/>
+      <c r="F2" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="61"/>
-      <c r="H2" s="64" t="s">
+      <c r="G2" s="48"/>
+      <c r="H2" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="64" t="s">
+      <c r="I2" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="62" t="s">
+      <c r="J2" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62"/>
-      <c r="N2" s="64" t="s">
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="62" t="s">
+      <c r="O2" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="P2" s="64" t="s">
+      <c r="P2" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="64"/>
-      <c r="R2" s="64"/>
+      <c r="Q2" s="51"/>
+      <c r="R2" s="51"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="33" t="s">
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="33" t="s">
+      <c r="K3" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L3" s="33" t="s">
+      <c r="L3" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="M3" s="33" t="s">
+      <c r="M3" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="N3" s="64"/>
-      <c r="O3" s="62"/>
-      <c r="P3" s="33" t="s">
+      <c r="N3" s="51"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="33" t="s">
+      <c r="Q3" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="33" t="s">
+      <c r="R3" s="19" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="29" t="str">
+      <c r="A4" s="15" t="str">
         <f>'Cabecera-Cpte'!E5</f>
         <v>B</v>
       </c>
-      <c r="B4" s="28">
+      <c r="B4" s="14">
         <f>'Cabecera-Cpte'!F5</f>
         <v>0</v>
       </c>
-      <c r="C4" s="28">
+      <c r="C4" s="14">
         <f>'Cabecera-Cpte'!G5</f>
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="str">
+      <c r="D4" s="15" t="str">
         <f>'Cabecera-Cpte'!O5</f>
         <v>CUI</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4" s="14">
         <f>'Cabecera-Cpte'!P5</f>
         <v>0</v>
       </c>
-      <c r="F4" s="34">
+      <c r="F4" s="20">
         <f>'Cabecera-Cpte'!K5</f>
         <v>0</v>
       </c>
-      <c r="G4" s="34">
+      <c r="G4" s="20">
         <f>'Cabecera-Cpte'!L5</f>
         <v>0</v>
       </c>
-      <c r="H4" s="29" t="s">
-        <v>157</v>
-      </c>
-      <c r="J4" s="29">
+      <c r="H4" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="J4" s="15">
         <v>3</v>
       </c>
-      <c r="K4" s="35">
+      <c r="K4" s="21">
         <v>1</v>
       </c>
-      <c r="L4" s="29">
+      <c r="L4" s="15">
         <v>1</v>
       </c>
-      <c r="M4" s="29">
+      <c r="M4" s="15">
         <v>0</v>
       </c>
-      <c r="N4" s="29">
+      <c r="N4" s="15">
         <v>1</v>
       </c>
-      <c r="P4" s="29">
+      <c r="P4" s="15">
         <f>'Cabecera-Cpte'!AI5</f>
         <v>0</v>
       </c>
@@ -5361,356 +4320,347 @@
   <dimension ref="A1:AJ4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="23" style="28" customWidth="1"/>
-    <col min="4" max="4" width="4.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23" style="29" customWidth="1"/>
-    <col min="6" max="7" width="23" style="28" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="29" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9" style="29" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="8.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="4" style="29" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8" style="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="4.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="6.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.7109375" style="29" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="23" style="29" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17.7109375" style="42" bestFit="1" customWidth="1"/>
-    <col min="37" max="16384" width="11.42578125" style="29"/>
+    <col min="1" max="1" width="5.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="23" style="14" customWidth="1"/>
+    <col min="4" max="4" width="4.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23" style="15" customWidth="1"/>
+    <col min="6" max="7" width="23" style="14" customWidth="1"/>
+    <col min="8" max="8" width="8.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6" style="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9" style="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="15" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="8.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5" style="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4" style="15" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="4" style="15" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="4.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8" style="15" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="4.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="6.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="23" style="15" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="17.7109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="37" max="16384" width="11.42578125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="43" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
-      <c r="Z1" s="43"/>
-      <c r="AA1" s="43"/>
-      <c r="AB1" s="43"/>
-      <c r="AC1" s="43"/>
-      <c r="AD1" s="43"/>
-      <c r="AE1" s="43"/>
-      <c r="AF1" s="43"/>
-      <c r="AG1" s="43"/>
-      <c r="AH1" s="43"/>
-      <c r="AI1" s="43"/>
-      <c r="AJ1" s="43"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="31"/>
+      <c r="Y1" s="31"/>
+      <c r="Z1" s="31"/>
+      <c r="AA1" s="31"/>
+      <c r="AB1" s="31"/>
+      <c r="AC1" s="31"/>
+      <c r="AD1" s="31"/>
+      <c r="AE1" s="31"/>
+      <c r="AF1" s="31"/>
+      <c r="AG1" s="31"/>
+      <c r="AH1" s="31"/>
+      <c r="AI1" s="31"/>
+      <c r="AJ1" s="31"/>
     </row>
     <row r="2" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45" t="s">
+      <c r="E2" s="29"/>
+      <c r="F2" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45" t="s">
+      <c r="G2" s="29"/>
+      <c r="H2" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="I2" s="45" t="s">
+      <c r="I2" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="J2" s="44" t="s">
+      <c r="J2" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44" t="s">
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="N2" s="44" t="s">
+      <c r="N2" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="44" t="s">
+      <c r="O2" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44"/>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
-      <c r="T2" s="44" t="s">
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="30"/>
+      <c r="S2" s="30"/>
+      <c r="T2" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="U2" s="44" t="s">
+      <c r="U2" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="V2" s="44"/>
-      <c r="W2" s="44"/>
-      <c r="X2" s="44"/>
-      <c r="Y2" s="45" t="s">
+      <c r="V2" s="30"/>
+      <c r="W2" s="30"/>
+      <c r="X2" s="30"/>
+      <c r="Y2" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="Z2" s="45" t="s">
+      <c r="Z2" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="AA2" s="45" t="s">
+      <c r="AA2" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="AB2" s="45" t="s">
+      <c r="AB2" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="AC2" s="45" t="s">
+      <c r="AC2" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="AD2" s="45" t="s">
+      <c r="AD2" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="AE2" s="45" t="s">
+      <c r="AE2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="AF2" s="45" t="s">
+      <c r="AF2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="AG2" s="45" t="s">
+      <c r="AG2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="AH2" s="45" t="s">
+      <c r="AH2" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="AI2" s="45" t="s">
+      <c r="AI2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="AJ2" s="65" t="s">
+      <c r="AJ2" s="32" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="30" t="s">
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="30" t="s">
+      <c r="K3" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="L3" s="30" t="s">
+      <c r="L3" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="29" t="s">
+      <c r="M3" s="30"/>
+      <c r="N3" s="30"/>
+      <c r="O3" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="P3" s="29" t="s">
+      <c r="P3" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="Q3" s="29" t="s">
+      <c r="Q3" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="R3" s="29" t="s">
+      <c r="R3" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="S3" s="29" t="s">
+      <c r="S3" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="T3" s="44"/>
-      <c r="U3" s="29" t="s">
+      <c r="T3" s="30"/>
+      <c r="U3" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="V3" s="29" t="s">
+      <c r="V3" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="W3" s="29" t="s">
+      <c r="W3" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="X3" s="29" t="s">
+      <c r="X3" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="45"/>
-      <c r="AA3" s="45"/>
-      <c r="AB3" s="45"/>
-      <c r="AC3" s="45"/>
-      <c r="AD3" s="45"/>
-      <c r="AE3" s="45"/>
-      <c r="AF3" s="45"/>
-      <c r="AG3" s="45"/>
-      <c r="AH3" s="45"/>
-      <c r="AI3" s="45"/>
-      <c r="AJ3" s="65"/>
+      <c r="Y3" s="29"/>
+      <c r="Z3" s="29"/>
+      <c r="AA3" s="29"/>
+      <c r="AB3" s="29"/>
+      <c r="AC3" s="29"/>
+      <c r="AD3" s="29"/>
+      <c r="AE3" s="29"/>
+      <c r="AF3" s="29"/>
+      <c r="AG3" s="29"/>
+      <c r="AH3" s="29"/>
+      <c r="AI3" s="29"/>
+      <c r="AJ3" s="32"/>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A4" s="29" t="str">
+      <c r="A4" s="15" t="str">
         <f>'Cabecera-Cpte'!E5</f>
         <v>B</v>
       </c>
-      <c r="B4" s="28">
+      <c r="B4" s="14">
         <f>'Cabecera-Cpte'!F5</f>
         <v>0</v>
       </c>
-      <c r="C4" s="28">
+      <c r="C4" s="14">
         <f>'Cabecera-Cpte'!G5</f>
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="str">
+      <c r="D4" s="15" t="str">
         <f>'Cabecera-Cpte'!O5</f>
         <v>CUI</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="15">
         <f>'Cabecera-Cpte'!P5</f>
         <v>0</v>
       </c>
-      <c r="F4" s="34">
+      <c r="F4" s="20">
         <f>'Cabecera-Cpte'!K5</f>
         <v>0</v>
       </c>
-      <c r="G4" s="34">
+      <c r="G4" s="20">
         <f>'Cabecera-Cpte'!L5</f>
         <v>0</v>
       </c>
-      <c r="J4" s="29">
+      <c r="J4" s="15">
         <v>41</v>
       </c>
-      <c r="K4" s="29">
+      <c r="K4" s="15">
         <v>4</v>
       </c>
-      <c r="L4" s="29">
+      <c r="L4" s="15">
         <v>0</v>
       </c>
-      <c r="M4" s="29">
+      <c r="M4" s="15">
         <f>'Cabecera-Cpte'!A5</f>
         <v>326</v>
       </c>
-      <c r="O4" s="29">
+      <c r="O4" s="15">
         <v>1</v>
       </c>
-      <c r="P4" s="29">
+      <c r="P4" s="15">
         <v>0</v>
       </c>
-      <c r="Q4" s="29">
+      <c r="Q4" s="15">
         <v>0</v>
       </c>
-      <c r="R4" s="29">
+      <c r="R4" s="15">
         <v>1</v>
       </c>
-      <c r="S4" s="29">
+      <c r="S4" s="15">
         <v>0</v>
       </c>
-      <c r="U4" s="29">
+      <c r="U4" s="15">
         <f>'Detalle Cpte FacGS'!J4</f>
         <v>3</v>
       </c>
-      <c r="V4" s="29">
+      <c r="V4" s="15">
         <f>'Detalle Cpte FacGS'!K4</f>
         <v>1</v>
       </c>
-      <c r="W4" s="29">
+      <c r="W4" s="15">
         <f>'Detalle Cpte FacGS'!L4</f>
         <v>1</v>
       </c>
-      <c r="X4" s="29">
+      <c r="X4" s="15">
         <f>'Detalle Cpte FacGS'!M4</f>
         <v>0</v>
       </c>
-      <c r="Y4" s="29">
+      <c r="Y4" s="15">
         <v>11</v>
       </c>
-      <c r="Z4" s="29">
+      <c r="Z4" s="15">
         <v>1</v>
       </c>
-      <c r="AB4" s="29">
+      <c r="AB4" s="15">
         <v>0</v>
       </c>
-      <c r="AC4" s="29">
+      <c r="AC4" s="15">
         <v>0</v>
       </c>
-      <c r="AE4" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF4" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="AG4" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="AH4" s="29">
+      <c r="AE4" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF4" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="AG4" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="AH4" s="15">
         <v>0</v>
       </c>
-      <c r="AJ4" s="42">
+      <c r="AJ4" s="28">
         <f>'Cabecera-Cpte'!AI5</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="AH2:AH3"/>
-    <mergeCell ref="O2:S2"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="U2:X2"/>
     <mergeCell ref="H1:AJ1"/>
     <mergeCell ref="Y2:Y3"/>
     <mergeCell ref="Z2:Z3"/>
@@ -5727,6 +4677,15 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="N2:N3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="AH2:AH3"/>
+    <mergeCell ref="O2:S2"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="U2:X2"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5754,42 +4713,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="69" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="52" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="53"/>
-      <c r="F2" s="52" t="s">
+      <c r="E2" s="40"/>
+      <c r="F2" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="71" t="s">
+      <c r="G2" s="40"/>
+      <c r="H2" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="67" t="s">
+      <c r="I2" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="67" t="s">
+      <c r="J2" s="53" t="s">
         <v>64</v>
       </c>
     </row>
@@ -5815,9 +4774,9 @@
       <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="72"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
@@ -5864,40 +4823,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="75" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="73" t="s">
+      <c r="I1" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="73"/>
+      <c r="J1" s="59"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="52" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="53"/>
-      <c r="F2" s="52" t="s">
+      <c r="E2" s="40"/>
+      <c r="F2" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="74"/>
-      <c r="J2" s="74"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -5921,7 +4880,7 @@
       <c r="G3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="76"/>
+      <c r="H3" s="62"/>
       <c r="I3" s="5" t="s">
         <v>33</v>
       </c>
@@ -5943,1391 +4902,4 @@
   <headerFooter alignWithMargins="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC4E742D-50D9-4649-81D4-D8D984D05528}">
-  <dimension ref="A3:L31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="87.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="13"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="15"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="G4" s="16"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="18"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="15"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="18"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="18"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="18"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="18"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G10" s="16"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="18"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="18"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G12" s="16"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="18"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="18"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="18"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="18"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G16" s="16"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="18"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="18"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G18" s="16"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="18"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G19" s="16"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="18"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G20" s="16"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="18"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G21" s="16"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="18"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G22" s="16"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="18"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G23" s="16"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="18"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G24" s="16"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="18"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G25" s="16"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="18"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G26" s="16"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="18"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G27" s="16"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="18"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="18"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G29" s="16"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="18"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G30" s="16"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="18"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="21"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E7CF3FB-17F2-47AE-9197-5D005A61D330}">
-  <dimension ref="A1:G27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="32.85546875" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" customWidth="1"/>
-    <col min="7" max="7" width="25.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12">
-        <v>1688</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
-        <v>1691</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
-        <v>3980</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
-        <v>5102</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
-        <v>9930</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" s="12">
-        <v>30645168794</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <v>12112</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D7" s="12">
-        <v>30571865684</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
-        <v>12188</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
-        <v>12700</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
-        <v>13239</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D10" s="12">
-        <v>30630467620</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
-        <v>24441</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
-        <v>48440</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
-        <v>69790</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D13" s="12">
-        <v>33689822989</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
-        <v>92132</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D14" s="12">
-        <v>30686692899</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
-        <v>125649</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
-        <v>153200</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D16" s="12">
-        <v>30707421041</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12">
-        <v>167215</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D17" s="12">
-        <v>30707919902</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
-        <v>173985</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D18" s="12">
-        <v>30672616774</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
-        <v>196990</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D19" s="12">
-        <v>30708617888</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12">
-        <v>250244</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12">
-        <v>250552</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
-        <v>316725</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12">
-        <v>344829</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12">
-        <v>374869</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="12">
-        <v>30711273197</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12">
-        <v>384417</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D25" s="12">
-        <v>30711513562</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
-        <v>490353</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12">
-        <v>594725</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D27" s="12">
-        <v>30715273906</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F27" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G27" s="12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>